<commit_message>
commit pricing and key driver uupgrades
</commit_message>
<xml_diff>
--- a/modules/keydriver/docs/templates/KeyDriver_Config_Template.xlsx
+++ b/modules/keydriver/docs/templates/KeyDriver_Config_Template.xlsx
@@ -10,12 +10,14 @@
     <sheet name="Variables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Segments" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="StatedImportance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CustomSlides" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Insights" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="269">
   <si>
     <t xml:space="preserve">TURAS Key Driver Analysis - Settings</t>
   </si>
@@ -504,6 +506,324 @@
   </si>
   <si>
     <t xml:space="preserve">[REQUIRED] Mean stated importance rating (1-10 scale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v10.4 FEATURES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_elastic_net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable Elastic Net regularized regression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elastic_net_alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elastic net mixing (0=ridge, 0.5=elastic net, 1=lasso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numeric between 0 and 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elastic_net_nfolds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-validation folds for lambda selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integer between 3 and 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_nca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable Necessary Condition Analysis (NCA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_dominance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable Dominance Analysis (Budescu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable_gam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable GAM nonlinear effects analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gam_k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis dimension for GAM smooth terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIAGNOSTICS THRESHOLDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vif_moderate_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIF threshold for moderate multicollinearity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numeric (default 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vif_high_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIF threshold for high multicollinearity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numeric (default 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTML SECTION VISIBILITY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_exec_summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Executive Summary section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_importance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Importance section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Method Comparison section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_effect_sizes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Effect Sizes section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_correlations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Correlation section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_quadrant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Quadrant section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_shap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show SHAP section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_diagnostics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Diagnostics section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_bootstrap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Bootstrap CI section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_segments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Segment Comparison section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">html_show_guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show Interpretation Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTML DISPLAY OPTIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">correlation_display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heatmap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation display mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heatmap or table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bootstrap_display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bootstrap display mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary or detailed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURAS Key Driver Analysis - Custom Slides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add qualitative commentary slides to the HTML report Pinned Views panel (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slide_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slide_content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slide_image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slide_order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Title displayed at top of slide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Slide body text (supports basic markdown)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Path to image file (PNG, JPG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Numeric sort order (default: sheet order)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURAS Key Driver Analysis - Insights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-populate analyst insights in the HTML report sections (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insight_text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image_path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Section key matching HTML report section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Analyst insight text to display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Path to image file for inline embedding (PNG, JPG, GIF, SVG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid Section Keys:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exec-summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Executive Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">importance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driver Importance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">method-comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method Comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">effect-sizes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effect Sizes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">correlations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlation Matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quadrant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importance-Performance Quadrant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shap-summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHAP Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diagnostics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagnostics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bootstrap-ci</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bootstrap CIs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">segment-comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment Comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elastic-net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elastic Net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Necessary Condition Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dominance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dominance Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nonlinear Effects (GAM)</t>
   </si>
 </sst>
 </file>
@@ -511,7 +831,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -521,35 +841,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FF323367"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF546E7A"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF323367"/>
       <name val="Calibri"/>
       <b/>
@@ -583,11 +874,46 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF546E7A"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF323367"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF37474F"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -601,17 +927,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F8E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFDE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F8E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -626,16 +957,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
+        <fgColor rgb="FFE3F2FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE3F2FD"/>
+        <fgColor rgb="FFD9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -671,61 +1007,74 @@
         <color rgb="FF323367"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1029,632 +1378,1042 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="14" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="13" t="s">
+      <c r="C10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="13" t="s">
+      <c r="C12" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="13" t="s">
+      <c r="C13" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="13" t="s">
+      <c r="C14" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15" s="13" t="s">
+      <c r="C15" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D16" s="13" t="s">
+      <c r="C16" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="C17" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="E17" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="13" t="s">
+      <c r="C19" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="13" t="s">
+      <c r="C20" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="13" t="s">
+      <c r="C21" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="13" t="s">
+      <c r="C22" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="6" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="13" t="s">
+      <c r="C23" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" s="6" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="11" t="n">
+      <c r="B24" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="C24" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="13" t="s">
+      <c r="C24" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="6" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="11" t="n">
+      <c r="B25" s="3" t="n">
         <v>1000</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="C25" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="13" t="s">
+      <c r="C26" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="13" t="s">
+      <c r="C27" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D28" s="13" t="s">
+      <c r="C28" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D30" s="13" t="s">
+      <c r="C30" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C31" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D31" s="13" t="s">
+      <c r="C31" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="6" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="s">
+      <c r="A32" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C32" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D32" s="13" t="s">
+      <c r="C32" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D33" s="13" t="s">
+      <c r="C33" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="E33" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="s">
+      <c r="A34" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C34" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34" s="13" t="s">
+      <c r="C34" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C35" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D35" s="13" t="s">
+      <c r="C35" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="s">
+      <c r="A36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C36" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D36" s="13" t="s">
+      <c r="C36" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="E36" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B38" s="11" t="n">
+      <c r="B38" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D38" s="13" t="s">
+      <c r="C38" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E38" s="14" t="s">
+      <c r="E38" s="6" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="11" t="n">
+      <c r="B39" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="C39" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" s="13" t="s">
+      <c r="C39" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E39" s="6" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="s">
+      <c r="A41" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C41" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D41" s="13" t="s">
+      <c r="C41" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="14" t="s">
+      <c r="E41" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="s">
+      <c r="A42" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C42" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D42" s="13" t="s">
+      <c r="C42" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D42" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E42" s="14" t="s">
+      <c r="E42" s="6" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="s">
+      <c r="A43" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C43" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D43" s="13" t="s">
+      <c r="C43" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D43" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="E43" s="14" t="s">
+      <c r="E43" s="6" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>164</v>
+      </c>
+      <c r="B46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" t="s">
+        <v>165</v>
+      </c>
+      <c r="E46" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>166</v>
+      </c>
+      <c r="B47" t="s">
+        <v>167</v>
+      </c>
+      <c r="C47" t="s">
+        <v>4</v>
+      </c>
+      <c r="D47" t="s">
+        <v>168</v>
+      </c>
+      <c r="E47" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B48" t="s">
+        <v>171</v>
+      </c>
+      <c r="C48" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" t="s">
+        <v>172</v>
+      </c>
+      <c r="E48" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>174</v>
+      </c>
+      <c r="B49" t="s">
+        <v>28</v>
+      </c>
+      <c r="C49" t="s">
+        <v>4</v>
+      </c>
+      <c r="D49" t="s">
+        <v>175</v>
+      </c>
+      <c r="E49" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>176</v>
+      </c>
+      <c r="B50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" t="s">
+        <v>4</v>
+      </c>
+      <c r="D50" t="s">
+        <v>177</v>
+      </c>
+      <c r="E50" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>178</v>
+      </c>
+      <c r="B51" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" t="s">
+        <v>179</v>
+      </c>
+      <c r="E51" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>180</v>
+      </c>
+      <c r="B52" t="s">
+        <v>181</v>
+      </c>
+      <c r="C52" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" t="s">
+        <v>182</v>
+      </c>
+      <c r="E52" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>184</v>
+      </c>
+      <c r="B54" t="s">
+        <v>181</v>
+      </c>
+      <c r="C54" t="s">
+        <v>4</v>
+      </c>
+      <c r="D54" t="s">
+        <v>185</v>
+      </c>
+      <c r="E54" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>187</v>
+      </c>
+      <c r="B55" t="s">
+        <v>171</v>
+      </c>
+      <c r="C55" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" t="s">
+        <v>188</v>
+      </c>
+      <c r="E55" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>191</v>
+      </c>
+      <c r="B57" t="s">
+        <v>81</v>
+      </c>
+      <c r="C57" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" t="s">
+        <v>192</v>
+      </c>
+      <c r="E57" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>193</v>
+      </c>
+      <c r="B58" t="s">
+        <v>81</v>
+      </c>
+      <c r="C58" t="s">
+        <v>4</v>
+      </c>
+      <c r="D58" t="s">
+        <v>194</v>
+      </c>
+      <c r="E58" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>195</v>
+      </c>
+      <c r="B59" t="s">
+        <v>81</v>
+      </c>
+      <c r="C59" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" t="s">
+        <v>196</v>
+      </c>
+      <c r="E59" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>197</v>
+      </c>
+      <c r="B60" t="s">
+        <v>81</v>
+      </c>
+      <c r="C60" t="s">
+        <v>4</v>
+      </c>
+      <c r="D60" t="s">
+        <v>198</v>
+      </c>
+      <c r="E60" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>199</v>
+      </c>
+      <c r="B61" t="s">
+        <v>81</v>
+      </c>
+      <c r="C61" t="s">
+        <v>4</v>
+      </c>
+      <c r="D61" t="s">
+        <v>200</v>
+      </c>
+      <c r="E61" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" t="s">
+        <v>81</v>
+      </c>
+      <c r="C62" t="s">
+        <v>4</v>
+      </c>
+      <c r="D62" t="s">
+        <v>202</v>
+      </c>
+      <c r="E62" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>203</v>
+      </c>
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" t="s">
+        <v>204</v>
+      </c>
+      <c r="E63" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>205</v>
+      </c>
+      <c r="B64" t="s">
+        <v>81</v>
+      </c>
+      <c r="C64" t="s">
+        <v>4</v>
+      </c>
+      <c r="D64" t="s">
+        <v>206</v>
+      </c>
+      <c r="E64" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B65" t="s">
+        <v>81</v>
+      </c>
+      <c r="C65" t="s">
+        <v>4</v>
+      </c>
+      <c r="D65" t="s">
+        <v>208</v>
+      </c>
+      <c r="E65" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>209</v>
+      </c>
+      <c r="B66" t="s">
+        <v>81</v>
+      </c>
+      <c r="C66" t="s">
+        <v>4</v>
+      </c>
+      <c r="D66" t="s">
+        <v>210</v>
+      </c>
+      <c r="E66" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>211</v>
+      </c>
+      <c r="B67" t="s">
+        <v>81</v>
+      </c>
+      <c r="C67" t="s">
+        <v>4</v>
+      </c>
+      <c r="D67" t="s">
+        <v>212</v>
+      </c>
+      <c r="E67" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="B68" s="18"/>
+      <c r="C68" s="18"/>
+      <c r="D68" s="18"/>
+      <c r="E68" s="18"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>214</v>
+      </c>
+      <c r="B69" t="s">
+        <v>215</v>
+      </c>
+      <c r="C69" t="s">
+        <v>4</v>
+      </c>
+      <c r="D69" t="s">
+        <v>216</v>
+      </c>
+      <c r="E69" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>218</v>
+      </c>
+      <c r="B70" t="s">
+        <v>219</v>
+      </c>
+      <c r="C70" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" t="s">
+        <v>220</v>
+      </c>
+      <c r="E70" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -1823,47 +2582,47 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="15" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="5" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1988,244 +2747,244 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row r="19">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
     </row>
     <row r="20">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
     </row>
     <row r="21">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row r="22">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
     </row>
     <row r="23">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
     </row>
     <row r="24">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
     </row>
     <row r="25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
     </row>
     <row r="26">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
     </row>
     <row r="27">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
     </row>
     <row r="28">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
     </row>
     <row r="29">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
     </row>
     <row r="30">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
     </row>
     <row r="31">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
     </row>
     <row r="32">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
     </row>
     <row r="33">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
     </row>
     <row r="34">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
     </row>
     <row r="35">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
     </row>
     <row r="36">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
     </row>
     <row r="37">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
     </row>
     <row r="38">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
     </row>
     <row r="39">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
     </row>
     <row r="40">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2277,29 +3036,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="9" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="15" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="5" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2326,54 +3085,54 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2400,23 +3159,23 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="9" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="15" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="5" t="s">
         <v>162</v>
       </c>
     </row>
@@ -2453,84 +3212,84 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
     </row>
     <row r="19">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
     </row>
     <row r="20">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
     </row>
     <row r="21">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
     </row>
     <row r="22">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
     </row>
     <row r="23">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
     </row>
     <row r="24">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
     </row>
     <row r="25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
     </row>
     <row r="26">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
     </row>
     <row r="27">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
     </row>
     <row r="28">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2546,4 +3305,235 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="20.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="50.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="25.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C4" t="s">
+        <v>230</v>
+      </c>
+      <c r="D4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="55.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="30.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>243</v>
+      </c>
+      <c r="B9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>247</v>
+      </c>
+      <c r="B11" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>253</v>
+      </c>
+      <c r="B14" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B15" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>257</v>
+      </c>
+      <c r="B16" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>259</v>
+      </c>
+      <c r="B17" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>263</v>
+      </c>
+      <c r="B19" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>265</v>
+      </c>
+      <c r="B20" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>267</v>
+      </c>
+      <c r="B21" t="s">
+        <v>268</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>